<commit_message>
Dashboard builder: example covenants at 1.20x lock-up and 1.00x default
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Ridgeline-Example-Inputs.xlsx
+++ b/dashboard-builder/Ridgeline-Example-Inputs.xlsx
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="B28" s="8">
-        <v>1.25</v>
+        <v>1.2</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="B29" s="8">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>

</xml_diff>